<commit_message>
add generic and case text elements to input xlsx for beerwiser (#37)
* add generic and case text elements to input xlsx for beerwiser

* add text files for other cases and formats

* add text files for other cases and formats

* Update pyproject.toml
</commit_message>
<xml_diff>
--- a/src/vlinder/data/DSM/xlsx/DSM.xlsx
+++ b/src/vlinder/data/DSM/xlsx/DSM.xlsx
@@ -1,37 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10414"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lheringa001\Desktop\RBS_opensource\trbs_dsm\model\data\DSM\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ttami001/Documents/forked_tbrs_opensource/trbs/src/vlinder/data/DSM/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47E91D93-C97C-46C5-A426-D7D1DDD1917D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CDD0B1E-C7CC-4C40-A40F-48BBBD72638E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="configurations" sheetId="1" r:id="rId1"/>
-    <sheet name="key_outputs" sheetId="2" r:id="rId2"/>
-    <sheet name="decision_makers_options" sheetId="3" r:id="rId3"/>
-    <sheet name="scenarios" sheetId="4" r:id="rId4"/>
-    <sheet name="fixed_inputs" sheetId="5" r:id="rId5"/>
-    <sheet name="dependencies" sheetId="7" r:id="rId6"/>
-    <sheet name="theme_weights" sheetId="8" r:id="rId7"/>
-    <sheet name="key_output_weights" sheetId="9" r:id="rId8"/>
-    <sheet name="scenario_weights" sheetId="10" r:id="rId9"/>
+    <sheet name="generic_text_elements" sheetId="11" r:id="rId2"/>
+    <sheet name="case_text_elements" sheetId="12" r:id="rId3"/>
+    <sheet name="key_outputs" sheetId="2" r:id="rId4"/>
+    <sheet name="decision_makers_options" sheetId="3" r:id="rId5"/>
+    <sheet name="scenarios" sheetId="4" r:id="rId6"/>
+    <sheet name="fixed_inputs" sheetId="5" r:id="rId7"/>
+    <sheet name="dependencies" sheetId="7" r:id="rId8"/>
+    <sheet name="theme_weights" sheetId="8" r:id="rId9"/>
+    <sheet name="key_output_weights" sheetId="9" r:id="rId10"/>
+    <sheet name="scenario_weights" sheetId="10" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">dependencies!$A$1:$H$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">dependencies!$A$1:$H$70</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="152">
   <si>
     <t>configuration</t>
   </si>
@@ -409,6 +411,84 @@
   </si>
   <si>
     <t>Total demand RS and RE</t>
+  </si>
+  <si>
+    <t>generic_text_element</t>
+  </si>
+  <si>
+    <t>title_strategic_challenge</t>
+  </si>
+  <si>
+    <t>Strategic Challenge</t>
+  </si>
+  <si>
+    <t>title_key_outputs</t>
+  </si>
+  <si>
+    <t>Key outputs</t>
+  </si>
+  <si>
+    <t>title_dmo</t>
+  </si>
+  <si>
+    <t>Options</t>
+  </si>
+  <si>
+    <t>title_scenarios</t>
+  </si>
+  <si>
+    <t>Scenarios</t>
+  </si>
+  <si>
+    <t>title_comparison</t>
+  </si>
+  <si>
+    <t>Comparisons of options</t>
+  </si>
+  <si>
+    <t>title_theme_weights</t>
+  </si>
+  <si>
+    <t>Key output and theme weights</t>
+  </si>
+  <si>
+    <t>title_scenario_weights</t>
+  </si>
+  <si>
+    <t>Scenario weights</t>
+  </si>
+  <si>
+    <t>text_strategic_challenge</t>
+  </si>
+  <si>
+    <t>Describing strategic challenge that requires a decision</t>
+  </si>
+  <si>
+    <t>text_key_outputs</t>
+  </si>
+  <si>
+    <t>Which indicators do you use to evaluate the impact of your decision(s)?</t>
+  </si>
+  <si>
+    <t>text_dmo</t>
+  </si>
+  <si>
+    <t>Which options do you have to influence your impact?</t>
+  </si>
+  <si>
+    <t>text_scenarios</t>
+  </si>
+  <si>
+    <t>Which uncertainty do you want to account for?</t>
+  </si>
+  <si>
+    <t>case_text_element</t>
+  </si>
+  <si>
+    <t>strategic_challenge</t>
+  </si>
+  <si>
+    <t>How to source energy?</t>
   </si>
 </sst>
 </file>
@@ -419,9 +499,16 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -431,6 +518,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -443,6 +531,7 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -460,17 +549,20 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -479,7 +571,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -489,6 +581,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -543,69 +641,71 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{AE53C5E1-75E6-4245-B0B1-466E5639B5C7}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -906,12 +1006,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -919,12 +1019,151 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="37.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="14">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="14">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -933,22 +1172,167 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2E1CC75-D97A-4B40-BEB4-D0908A445A81}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="21.6640625" style="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="163.5" style="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="21" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="21" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="21" t="s">
+        <v>135</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="21" t="s">
+        <v>143</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="21" t="s">
+        <v>145</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="21" t="s">
+        <v>147</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>148</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA2AD5AE-B0E9-A747-915F-4F9B572E98DB}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.1640625" style="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" style="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="20" t="s">
+        <v>150</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B3" s="21"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -977,248 +1361,239 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>31</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="13">
+      <c r="C2">
         <v>0</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
       </c>
-      <c r="E2" s="13">
-        <v>0</v>
-      </c>
-      <c r="F2" s="13">
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
         <v>1</v>
       </c>
-      <c r="G2" s="14">
+      <c r="G2" s="13">
         <v>-41400000</v>
       </c>
-      <c r="H2" s="14">
+      <c r="H2" s="13">
         <v>30000000</v>
       </c>
-      <c r="I2" s="13"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>32</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3">
         <v>0</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>
       </c>
-      <c r="E3" s="13">
+      <c r="E3">
         <v>1</v>
       </c>
-      <c r="F3" s="13">
+      <c r="F3">
         <v>1</v>
       </c>
-      <c r="G3" s="14">
+      <c r="G3" s="13">
         <v>5734800</v>
       </c>
-      <c r="H3" s="14">
+      <c r="H3" s="13">
         <v>8389800</v>
       </c>
-      <c r="I3" s="13"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
         <v>33</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4">
         <v>0</v>
       </c>
       <c r="D4" s="3">
         <v>0</v>
       </c>
-      <c r="E4" s="13">
-        <v>0</v>
-      </c>
-      <c r="F4" s="13">
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
         <v>1</v>
       </c>
-      <c r="G4" s="14">
-        <v>0</v>
-      </c>
-      <c r="H4" s="14">
+      <c r="G4" s="13">
+        <v>0</v>
+      </c>
+      <c r="H4" s="13">
         <v>0.1</v>
       </c>
-      <c r="I4" s="13"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>34</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5">
         <v>0</v>
       </c>
       <c r="D5" s="3">
         <v>0</v>
       </c>
-      <c r="E5" s="13">
-        <v>0</v>
-      </c>
-      <c r="F5" s="13">
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
         <v>1</v>
       </c>
-      <c r="G5" s="14">
-        <v>0</v>
-      </c>
-      <c r="H5" s="14">
+      <c r="G5" s="13">
+        <v>0</v>
+      </c>
+      <c r="H5" s="13">
         <v>3988.3999999999942</v>
       </c>
-      <c r="I5" s="13"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>35</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6">
         <v>0</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
       </c>
-      <c r="E6" s="13">
-        <v>0</v>
-      </c>
-      <c r="F6" s="13">
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
         <v>1</v>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="13">
         <v>39884</v>
       </c>
-      <c r="H6" s="14">
+      <c r="H6" s="13">
         <v>39884</v>
       </c>
-      <c r="I6" s="13"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
         <v>36</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7">
         <v>0</v>
       </c>
       <c r="D7" s="3">
         <v>0</v>
       </c>
-      <c r="E7" s="13">
-        <v>0</v>
-      </c>
-      <c r="F7" s="13">
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
         <v>1</v>
       </c>
-      <c r="G7" s="14">
-        <v>0</v>
-      </c>
-      <c r="H7" s="14">
+      <c r="G7" s="13">
+        <v>0</v>
+      </c>
+      <c r="H7" s="13">
         <v>1.73</v>
       </c>
-      <c r="I7" s="13"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
         <v>37</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8">
         <v>0</v>
       </c>
       <c r="D8" s="3">
         <v>0</v>
       </c>
-      <c r="E8" s="13">
-        <v>0</v>
-      </c>
-      <c r="F8" s="13">
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
         <v>1</v>
       </c>
-      <c r="G8" s="14">
-        <v>0</v>
-      </c>
-      <c r="H8" s="14">
+      <c r="G8" s="13">
+        <v>0</v>
+      </c>
+      <c r="H8" s="13">
         <v>1.1244999999999998</v>
       </c>
-      <c r="I8" s="13"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
         <v>38</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9">
         <v>0</v>
       </c>
       <c r="D9" s="3">
         <v>0</v>
       </c>
-      <c r="E9" s="13">
-        <v>0</v>
-      </c>
-      <c r="F9" s="13">
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
         <v>1</v>
       </c>
-      <c r="G9" s="14">
-        <v>0</v>
-      </c>
-      <c r="H9" s="14">
+      <c r="G9" s="13">
+        <v>0</v>
+      </c>
+      <c r="H9" s="13">
         <v>0.17300000000000001</v>
       </c>
-      <c r="I9" s="13"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
         <v>39</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10">
         <v>0</v>
       </c>
       <c r="D10" s="3">
         <v>0</v>
       </c>
-      <c r="E10" s="13">
-        <v>0</v>
-      </c>
-      <c r="F10" s="13">
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
         <v>1</v>
       </c>
-      <c r="G10" s="14">
-        <v>0</v>
-      </c>
-      <c r="H10" s="14">
+      <c r="G10" s="13">
+        <v>0</v>
+      </c>
+      <c r="H10" s="13">
         <v>845540.79999999877</v>
       </c>
-      <c r="I10" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1226,16 +1601,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -1246,7 +1621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>40</v>
       </c>
@@ -1257,7 +1632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>43</v>
       </c>
@@ -1268,7 +1643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>41</v>
       </c>
@@ -1279,7 +1654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>42</v>
       </c>
@@ -1290,7 +1665,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>111</v>
       </c>
@@ -1301,7 +1676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>110</v>
       </c>
@@ -1312,7 +1687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>112</v>
       </c>
@@ -1323,7 +1698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
@@ -1334,7 +1709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>43</v>
       </c>
@@ -1345,7 +1720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>41</v>
       </c>
@@ -1356,7 +1731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>42</v>
       </c>
@@ -1367,7 +1742,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>111</v>
       </c>
@@ -1378,7 +1753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>110</v>
       </c>
@@ -1389,7 +1764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>112</v>
       </c>
@@ -1400,7 +1775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>40</v>
       </c>
@@ -1411,7 +1786,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>43</v>
       </c>
@@ -1422,7 +1797,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>41</v>
       </c>
@@ -1433,7 +1808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>42</v>
       </c>
@@ -1444,7 +1819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>111</v>
       </c>
@@ -1455,7 +1830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>110</v>
       </c>
@@ -1466,7 +1841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>112</v>
       </c>
@@ -1477,7 +1852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>40</v>
       </c>
@@ -1488,7 +1863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>43</v>
       </c>
@@ -1499,7 +1874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>41</v>
       </c>
@@ -1510,7 +1885,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>42</v>
       </c>
@@ -1521,7 +1896,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>111</v>
       </c>
@@ -1532,7 +1907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>110</v>
       </c>
@@ -1543,7 +1918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>112</v>
       </c>
@@ -1554,7 +1929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>40</v>
       </c>
@@ -1565,7 +1940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>43</v>
       </c>
@@ -1576,7 +1951,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>41</v>
       </c>
@@ -1587,7 +1962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>42</v>
       </c>
@@ -1598,7 +1973,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>111</v>
       </c>
@@ -1609,7 +1984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>110</v>
       </c>
@@ -1620,7 +1995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>112</v>
       </c>
@@ -1631,7 +2006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>40</v>
       </c>
@@ -1643,7 +2018,7 @@
       </c>
       <c r="F37" s="10"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>43</v>
       </c>
@@ -1655,7 +2030,7 @@
       </c>
       <c r="F38" s="10"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>41</v>
       </c>
@@ -1667,7 +2042,7 @@
       </c>
       <c r="F39" s="10"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>42</v>
       </c>
@@ -1679,7 +2054,7 @@
       </c>
       <c r="F40" s="10"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>111</v>
       </c>
@@ -1691,7 +2066,7 @@
       </c>
       <c r="F41" s="10"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>110</v>
       </c>
@@ -1703,7 +2078,7 @@
       </c>
       <c r="F42" s="10"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>112</v>
       </c>
@@ -1723,17 +2098,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
@@ -1744,7 +2119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>48</v>
       </c>
@@ -1755,7 +2130,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>49</v>
       </c>
@@ -1766,7 +2141,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>50</v>
       </c>
@@ -1777,7 +2152,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>51</v>
       </c>
@@ -1788,7 +2163,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>52</v>
       </c>
@@ -1799,7 +2174,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>53</v>
       </c>
@@ -1810,7 +2185,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>54</v>
       </c>
@@ -1821,7 +2196,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>48</v>
       </c>
@@ -1832,7 +2207,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>49</v>
       </c>
@@ -1843,7 +2218,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>50</v>
       </c>
@@ -1854,7 +2229,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
         <v>51</v>
       </c>
@@ -1865,7 +2240,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
         <v>52</v>
       </c>
@@ -1876,7 +2251,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
         <v>53</v>
       </c>
@@ -1887,7 +2262,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
         <v>54</v>
       </c>
@@ -1898,7 +2273,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
         <v>48</v>
       </c>
@@ -1909,7 +2284,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
         <v>49</v>
       </c>
@@ -1920,7 +2295,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
         <v>50</v>
       </c>
@@ -1931,7 +2306,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
         <v>51</v>
       </c>
@@ -1942,7 +2317,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
         <v>52</v>
       </c>
@@ -1953,7 +2328,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
         <v>53</v>
       </c>
@@ -1964,7 +2339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
         <v>54</v>
       </c>
@@ -1980,15 +2355,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B71"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="61.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="61.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
@@ -1996,7 +2371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>57</v>
       </c>
@@ -2004,7 +2379,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>58</v>
       </c>
@@ -2012,7 +2387,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>59</v>
       </c>
@@ -2020,7 +2395,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>60</v>
       </c>
@@ -2028,7 +2403,7 @@
         <v>0.67600000000000005</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>61</v>
       </c>
@@ -2036,7 +2411,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>62</v>
       </c>
@@ -2044,7 +2419,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>63</v>
       </c>
@@ -2052,7 +2427,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>64</v>
       </c>
@@ -2060,7 +2435,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>65</v>
       </c>
@@ -2068,7 +2443,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>66</v>
       </c>
@@ -2076,7 +2451,7 @@
         <v>1.7299999999999999E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>67</v>
       </c>
@@ -2084,7 +2459,7 @@
         <v>1.7299999999999999E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>68</v>
       </c>
@@ -2092,7 +2467,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>69</v>
       </c>
@@ -2100,7 +2475,7 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>70</v>
       </c>
@@ -2108,172 +2483,172 @@
         <v>40000000</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="7"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="7"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="7"/>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="7"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="7"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" s="7"/>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="7"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" s="7"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" s="7"/>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" s="7"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" s="7"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" s="7"/>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" s="7"/>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" s="7"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" s="7"/>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" s="7"/>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" s="7"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" s="7"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" s="7"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" s="7"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" s="7"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" s="7"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" s="7"/>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" s="7"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" s="7"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" s="7"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" s="7"/>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" s="7"/>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" s="7"/>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" s="7"/>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" s="7"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A47" s="7"/>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" s="7"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" s="7"/>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" s="7"/>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" s="7"/>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" s="7"/>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" s="7"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A54" s="7"/>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" s="7"/>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A56" s="7"/>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" s="7"/>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A58" s="7"/>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A59" s="7"/>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A60" s="7"/>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A61" s="7"/>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A62" s="7"/>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A63" s="7"/>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A64" s="7"/>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A65" s="7"/>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A66" s="7"/>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A67" s="7"/>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A68" s="7"/>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A69" s="7"/>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A70" s="7"/>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A71" s="7"/>
     </row>
   </sheetData>
@@ -2281,22 +2656,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H72"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="67.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="67.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
@@ -2322,7 +2697,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
         <v>71</v>
       </c>
@@ -2336,7 +2711,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>71</v>
       </c>
@@ -2350,7 +2725,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
         <v>72</v>
       </c>
@@ -2364,7 +2739,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>73</v>
       </c>
@@ -2378,49 +2753,49 @@
         <v>118</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="11" t="s">
         <v>73</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>124</v>
       </c>
       <c r="B7" s="11">
         <v>1</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" t="s">
         <v>54</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>124</v>
       </c>
       <c r="B8" s="11">
         <v>0</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" t="s">
         <v>53</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="17" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>74</v>
       </c>
@@ -2434,7 +2809,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>103</v>
       </c>
@@ -2448,21 +2823,21 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="17" t="s">
         <v>124</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
         <v>75</v>
       </c>
@@ -2476,7 +2851,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
         <v>76</v>
       </c>
@@ -2490,7 +2865,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>77</v>
       </c>
@@ -2504,7 +2879,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
         <v>78</v>
       </c>
@@ -2518,7 +2893,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
         <v>79</v>
       </c>
@@ -2532,7 +2907,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
         <v>80</v>
       </c>
@@ -2546,7 +2921,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
         <v>81</v>
       </c>
@@ -2560,7 +2935,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
         <v>82</v>
       </c>
@@ -2574,7 +2949,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
         <v>83</v>
       </c>
@@ -2588,7 +2963,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
         <v>84</v>
       </c>
@@ -2602,7 +2977,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
         <v>85</v>
       </c>
@@ -2616,7 +2991,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
         <v>86</v>
       </c>
@@ -2630,7 +3005,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
         <v>87</v>
       </c>
@@ -2644,7 +3019,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>88</v>
       </c>
@@ -2658,7 +3033,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
         <v>88</v>
       </c>
@@ -2672,7 +3047,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
         <v>89</v>
       </c>
@@ -2686,7 +3061,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
         <v>90</v>
       </c>
@@ -2700,7 +3075,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
         <v>91</v>
       </c>
@@ -2714,7 +3089,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="11" t="s">
         <v>91</v>
       </c>
@@ -2728,7 +3103,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="11" t="s">
         <v>125</v>
       </c>
@@ -2742,7 +3117,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="11" t="s">
         <v>125</v>
       </c>
@@ -2756,7 +3131,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="11" t="s">
         <v>125</v>
       </c>
@@ -2770,21 +3145,21 @@
         <v>121</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="11" t="s">
         <v>93</v>
       </c>
       <c r="B34" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C34" s="20" t="s">
+      <c r="C34" s="18" t="s">
         <v>125</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="11" t="s">
         <v>94</v>
       </c>
@@ -2798,7 +3173,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="11" t="s">
         <v>104</v>
       </c>
@@ -2812,7 +3187,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="11" t="s">
         <v>104</v>
       </c>
@@ -2826,7 +3201,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="11" t="s">
         <v>105</v>
       </c>
@@ -2840,7 +3215,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="11" t="s">
         <v>106</v>
       </c>
@@ -2854,7 +3229,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="11" t="s">
         <v>106</v>
       </c>
@@ -2868,7 +3243,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="11" t="s">
         <v>107</v>
       </c>
@@ -2882,7 +3257,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="11" t="s">
         <v>95</v>
       </c>
@@ -2896,7 +3271,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="11" t="s">
         <v>95</v>
       </c>
@@ -2910,7 +3285,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="11" t="s">
         <v>96</v>
       </c>
@@ -2924,7 +3299,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="11" t="s">
         <v>35</v>
       </c>
@@ -2938,7 +3313,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="11" t="s">
         <v>97</v>
       </c>
@@ -2952,7 +3327,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="11" t="s">
         <v>32</v>
       </c>
@@ -2966,7 +3341,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="11" t="s">
         <v>32</v>
       </c>
@@ -2980,7 +3355,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="11" t="s">
         <v>32</v>
       </c>
@@ -2994,7 +3369,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="11" t="s">
         <v>33</v>
       </c>
@@ -3008,7 +3383,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="11" t="s">
         <v>33</v>
       </c>
@@ -3022,7 +3397,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="11" t="s">
         <v>98</v>
       </c>
@@ -3036,7 +3411,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" s="11" t="s">
         <v>34</v>
       </c>
@@ -3050,7 +3425,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="11" t="s">
         <v>34</v>
       </c>
@@ -3064,21 +3439,21 @@
         <v>120</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="16" t="s">
+    <row r="55" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A55" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B55" s="16" t="s">
+      <c r="B55" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C55" s="16" t="s">
+      <c r="C55" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="D55" s="16" t="s">
+      <c r="D55" s="15" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="11" t="s">
         <v>100</v>
       </c>
@@ -3092,149 +3467,149 @@
         <v>115</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="16" t="s">
+    <row r="57" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A57" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="B57" s="16" t="s">
+      <c r="B57" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="C57" s="16" t="s">
+      <c r="C57" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="D57" s="16" t="s">
+      <c r="D57" s="15" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="16" t="s">
+    <row r="58" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A58" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="B58" s="16" t="s">
+      <c r="B58" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="C58" s="16" t="s">
+      <c r="C58" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D58" s="16" t="s">
+      <c r="D58" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="E58" s="17"/>
-      <c r="F58" s="17"/>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="16" t="s">
+      <c r="E58" s="16"/>
+      <c r="F58" s="16"/>
+    </row>
+    <row r="59" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A59" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="B59" s="16">
+      <c r="B59" s="15">
         <v>1</v>
       </c>
-      <c r="C59" s="16" t="s">
+      <c r="C59" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="D59" s="16" t="s">
+      <c r="D59" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="E59" s="17"/>
-      <c r="F59" s="17"/>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="16" t="s">
+      <c r="E59" s="16"/>
+      <c r="F59" s="16"/>
+    </row>
+    <row r="60" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A60" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="B60" s="16">
+      <c r="B60" s="15">
         <v>1</v>
       </c>
-      <c r="C60" s="16" t="s">
+      <c r="C60" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="D60" s="16" t="s">
+      <c r="D60" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="E60" s="17"/>
-      <c r="F60" s="17"/>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="16" t="s">
+      <c r="E60" s="16"/>
+      <c r="F60" s="16"/>
+    </row>
+    <row r="61" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A61" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B61" s="16" t="s">
+      <c r="B61" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="C61" s="16" t="s">
+      <c r="C61" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D61" s="16" t="s">
+      <c r="D61" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E61" s="17"/>
-      <c r="F61" s="17"/>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="16" t="s">
+      <c r="E61" s="16"/>
+      <c r="F61" s="16"/>
+    </row>
+    <row r="62" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A62" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="B62" s="16" t="s">
+      <c r="B62" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="C62" s="16" t="s">
+      <c r="C62" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="D62" s="16" t="s">
+      <c r="D62" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E62" s="17"/>
-      <c r="F62" s="17"/>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="16" t="s">
+      <c r="E62" s="16"/>
+      <c r="F62" s="16"/>
+    </row>
+    <row r="63" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A63" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="B63" s="16" t="s">
+      <c r="B63" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="C63" s="16" t="s">
+      <c r="C63" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D63" s="16" t="s">
+      <c r="D63" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E63" s="17"/>
-      <c r="F63" s="17"/>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="16" t="s">
+      <c r="E63" s="16"/>
+      <c r="F63" s="16"/>
+    </row>
+    <row r="64" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A64" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="B64" s="16" t="s">
+      <c r="B64" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="C64" s="16" t="s">
+      <c r="C64" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="D64" s="16" t="s">
+      <c r="D64" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E64" s="17"/>
-      <c r="F64" s="17"/>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="16" t="s">
+      <c r="E64" s="16"/>
+      <c r="F64" s="16"/>
+    </row>
+    <row r="65" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A65" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B65" s="16" t="s">
+      <c r="B65" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="C65" s="16" t="s">
+      <c r="C65" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="D65" s="16" t="s">
+      <c r="D65" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="E65" s="17"/>
-      <c r="F65" s="17"/>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E65" s="16"/>
+      <c r="F65" s="16"/>
+    </row>
+    <row r="66" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="11" t="s">
         <v>99</v>
       </c>
@@ -3247,11 +3622,11 @@
       <c r="D66" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="E66" s="17"/>
-      <c r="F66" s="17"/>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" s="16" t="s">
+      <c r="E66" s="16"/>
+      <c r="F66" s="16"/>
+    </row>
+    <row r="67" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A67" s="15" t="s">
         <v>102</v>
       </c>
       <c r="B67" s="11" t="s">
@@ -3263,56 +3638,56 @@
       <c r="D67" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="E67" s="17"/>
-      <c r="F67" s="17"/>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="16" t="s">
+      <c r="E67" s="16"/>
+      <c r="F67" s="16"/>
+    </row>
+    <row r="68" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A68" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="B68" s="16">
-        <v>0</v>
-      </c>
-      <c r="C68" s="16" t="s">
+      <c r="B68" s="15">
+        <v>0</v>
+      </c>
+      <c r="C68" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="D68" s="16" t="s">
+      <c r="D68" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E68" s="17"/>
-      <c r="F68" s="17"/>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="16" t="s">
+      <c r="E68" s="16"/>
+      <c r="F68" s="16"/>
+    </row>
+    <row r="69" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A69" s="15" t="s">
         <v>102</v>
       </c>
       <c r="B69">
         <v>0</v>
       </c>
-      <c r="C69" s="16" t="s">
+      <c r="C69" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="D69" s="16" t="s">
+      <c r="D69" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="E69" s="17"/>
-      <c r="F69" s="17"/>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E70" s="17"/>
-      <c r="F70" s="17"/>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E71" s="17"/>
-      <c r="F71" s="17"/>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" s="17"/>
-      <c r="B72" s="17"/>
-      <c r="C72" s="17"/>
-      <c r="D72" s="17"/>
-      <c r="E72" s="17"/>
-      <c r="F72" s="17"/>
+      <c r="E69" s="16"/>
+      <c r="F69" s="16"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E70" s="16"/>
+      <c r="F70" s="16"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E71" s="16"/>
+      <c r="F71" s="16"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A72" s="16"/>
+      <c r="B72" s="16"/>
+      <c r="C72" s="16"/>
+      <c r="D72" s="16"/>
+      <c r="E72" s="16"/>
+      <c r="F72" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3320,12 +3695,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -3333,7 +3708,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -3341,7 +3716,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -3349,150 +3724,11 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>14</v>
       </c>
       <c r="B4">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B4" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="B8" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="B9" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="B10" s="15">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="B2" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="B4" s="15">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix demo cases and warnings (#106)
Co-authored-by: Thom-Ivar van Dijk <thomivar@gmail.com>
</commit_message>
<xml_diff>
--- a/src/vlinder/data/DSM/xlsx/DSM.xlsx
+++ b/src/vlinder/data/DSM/xlsx/DSM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tdijk004/Documents/Tooling/vlinder/trbs/src/vlinder/data/DSM/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C96E510B-52E3-F148-9B58-550F0A72945F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{114CF110-45FB-9346-9CA8-CB0A11CEA40D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19800" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19800" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="configurations" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="181">
   <si>
     <t>configuration</t>
   </si>
@@ -201,9 +201,6 @@
   </si>
   <si>
     <t>Current employee engagement score</t>
-  </si>
-  <si>
-    <t>Current Net Promotor Score</t>
   </si>
   <si>
     <t>Disengaged employee recommendation rate</t>
@@ -1129,10 +1126,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B2" t="s">
         <v>180</v>
-      </c>
-      <c r="B2" t="s">
-        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -1252,7 +1249,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" s="14">
         <v>1</v>
@@ -1291,7 +1288,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="18" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B1" s="18" t="s">
         <v>1</v>
@@ -1299,238 +1296,238 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="20" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3" s="20" t="s">
         <v>121</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="B4" s="20" t="s">
         <v>123</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="20" t="s">
+        <v>124</v>
+      </c>
+      <c r="B5" s="20" t="s">
         <v>125</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="B6" s="20" t="s">
         <v>134</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="B7" s="20" t="s">
         <v>136</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="B8" s="21" t="s">
         <v>138</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="B9" s="21" t="s">
         <v>140</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="B10" s="21" t="s">
         <v>142</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="20" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="20" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="20" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="20" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="20" t="s">
+        <v>147</v>
+      </c>
+      <c r="B15" s="20" t="s">
         <v>148</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="20" t="s">
+        <v>149</v>
+      </c>
+      <c r="B16" s="20" t="s">
         <v>150</v>
-      </c>
-      <c r="B16" s="20" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="B17" s="21" t="s">
         <v>152</v>
-      </c>
-      <c r="B17" s="21" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="B18" s="20" t="s">
         <v>154</v>
-      </c>
-      <c r="B18" s="20" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="B19" s="20" t="s">
         <v>156</v>
-      </c>
-      <c r="B19" s="20" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="20" t="s">
+        <v>157</v>
+      </c>
+      <c r="B20" s="20" t="s">
         <v>158</v>
-      </c>
-      <c r="B20" s="20" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B21" s="20"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B22" s="20"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="B23" s="20" t="s">
         <v>162</v>
-      </c>
-      <c r="B23" s="20" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="B24" s="20" t="s">
         <v>164</v>
-      </c>
-      <c r="B24" s="20" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="B25" s="20" t="s">
         <v>166</v>
-      </c>
-      <c r="B25" s="20" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="B26" s="20" t="s">
         <v>168</v>
-      </c>
-      <c r="B26" s="20" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" s="20" t="s">
+        <v>169</v>
+      </c>
+      <c r="B27" s="20" t="s">
         <v>170</v>
-      </c>
-      <c r="B27" s="20" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="B28" s="20" t="s">
         <v>172</v>
-      </c>
-      <c r="B28" s="20" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="20" t="s">
+        <v>173</v>
+      </c>
+      <c r="B29" s="20" t="s">
         <v>174</v>
-      </c>
-      <c r="B29" s="20" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="B30" s="20" t="s">
         <v>176</v>
-      </c>
-      <c r="B30" s="20" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="20" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -1550,7 +1547,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B1" s="18" t="s">
         <v>1</v>
@@ -1558,10 +1555,10 @@
     </row>
     <row r="2" spans="1:2" ht="204" x14ac:dyDescent="0.2">
       <c r="A2" s="19" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -1632,12 +1629,8 @@
       <c r="F2">
         <v>1</v>
       </c>
-      <c r="G2" s="13">
-        <v>-41400000</v>
-      </c>
-      <c r="H2" s="13">
-        <v>30000000</v>
-      </c>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
@@ -1658,12 +1651,8 @@
       <c r="F3">
         <v>1</v>
       </c>
-      <c r="G3" s="13">
-        <v>5734800</v>
-      </c>
-      <c r="H3" s="13">
-        <v>8389800</v>
-      </c>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
@@ -1684,12 +1673,8 @@
       <c r="F4">
         <v>1</v>
       </c>
-      <c r="G4" s="13">
-        <v>0</v>
-      </c>
-      <c r="H4" s="13">
-        <v>0.1</v>
-      </c>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
@@ -1710,12 +1695,8 @@
       <c r="F5">
         <v>1</v>
       </c>
-      <c r="G5" s="13">
-        <v>0</v>
-      </c>
-      <c r="H5" s="13">
-        <v>3988.3999999999942</v>
-      </c>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
@@ -1736,12 +1717,8 @@
       <c r="F6">
         <v>1</v>
       </c>
-      <c r="G6" s="13">
-        <v>39884</v>
-      </c>
-      <c r="H6" s="13">
-        <v>39884</v>
-      </c>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
@@ -1762,12 +1739,8 @@
       <c r="F7">
         <v>1</v>
       </c>
-      <c r="G7" s="13">
-        <v>0</v>
-      </c>
-      <c r="H7" s="13">
-        <v>1.73</v>
-      </c>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
@@ -1788,12 +1761,8 @@
       <c r="F8">
         <v>1</v>
       </c>
-      <c r="G8" s="13">
-        <v>0</v>
-      </c>
-      <c r="H8" s="13">
-        <v>1.1244999999999998</v>
-      </c>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
@@ -1814,12 +1783,8 @@
       <c r="F9">
         <v>1</v>
       </c>
-      <c r="G9" s="13">
-        <v>0</v>
-      </c>
-      <c r="H9" s="13">
-        <v>0.17300000000000001</v>
-      </c>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
@@ -1840,12 +1805,8 @@
       <c r="F10">
         <v>1</v>
       </c>
-      <c r="G10" s="13">
-        <v>0</v>
-      </c>
-      <c r="H10" s="13">
-        <v>845540.79999999877</v>
-      </c>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1878,7 +1839,7 @@
         <v>34</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C2" s="5">
         <v>0</v>
@@ -1889,7 +1850,7 @@
         <v>37</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C3" s="5">
         <v>0</v>
@@ -1900,7 +1861,7 @@
         <v>35</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C4" s="5">
         <v>0</v>
@@ -1911,7 +1872,7 @@
         <v>36</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C5" s="5">
         <v>0</v>
@@ -1919,10 +1880,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C6" s="5">
         <v>0</v>
@@ -1930,10 +1891,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C7" s="5">
         <v>0</v>
@@ -1941,10 +1902,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C8" s="5">
         <v>0</v>
@@ -1996,7 +1957,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>40</v>
@@ -2007,7 +1968,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>40</v>
@@ -2018,7 +1979,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>40</v>
@@ -2032,7 +1993,7 @@
         <v>34</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C16" s="5">
         <v>0</v>
@@ -2043,7 +2004,7 @@
         <v>37</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C17" s="5">
         <v>0.5</v>
@@ -2054,7 +2015,7 @@
         <v>35</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C18" s="5">
         <v>0</v>
@@ -2065,7 +2026,7 @@
         <v>36</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C19" s="5">
         <v>0</v>
@@ -2073,10 +2034,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C20" s="5">
         <v>0</v>
@@ -2084,10 +2045,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C21" s="5">
         <v>0</v>
@@ -2095,10 +2056,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C22" s="5">
         <v>0</v>
@@ -2150,7 +2111,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>39</v>
@@ -2161,7 +2122,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>39</v>
@@ -2172,7 +2133,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>39</v>
@@ -2227,7 +2188,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>41</v>
@@ -2238,7 +2199,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>41</v>
@@ -2249,7 +2210,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>41</v>
@@ -2308,7 +2269,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>38</v>
@@ -2320,7 +2281,7 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>38</v>
@@ -2332,7 +2293,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>38</v>
@@ -2376,7 +2337,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C2" s="6">
         <v>108</v>
@@ -2387,7 +2348,7 @@
         <v>43</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C3" s="6">
         <v>270</v>
@@ -2398,7 +2359,7 @@
         <v>44</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C4" s="6">
         <v>130</v>
@@ -2409,7 +2370,7 @@
         <v>45</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C5" s="6">
         <v>115</v>
@@ -2420,7 +2381,7 @@
         <v>46</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C6" s="6">
         <v>51</v>
@@ -2431,7 +2392,7 @@
         <v>47</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C7" s="6">
         <v>0.3</v>
@@ -2442,7 +2403,7 @@
         <v>48</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C8" s="6">
         <v>0.3</v>
@@ -2609,7 +2570,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:B71"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="61.5" bestFit="1" customWidth="1"/>
@@ -2668,7 +2629,7 @@
         <v>56</v>
       </c>
       <c r="B7" s="8">
-        <v>0.36</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -2676,7 +2637,7 @@
         <v>57</v>
       </c>
       <c r="B8" s="8">
-        <v>0.13</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -2684,7 +2645,7 @@
         <v>58</v>
       </c>
       <c r="B9" s="8">
-        <v>212</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -2692,7 +2653,7 @@
         <v>59</v>
       </c>
       <c r="B10" s="8">
-        <v>0.1</v>
+        <v>1.7299999999999999E-2</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -2708,7 +2669,7 @@
         <v>61</v>
       </c>
       <c r="B12" s="8">
-        <v>1.7299999999999999E-2</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -2716,7 +2677,7 @@
         <v>62</v>
       </c>
       <c r="B13" s="8">
-        <v>30000</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -2724,16 +2685,11 @@
         <v>63</v>
       </c>
       <c r="B14" s="8">
-        <v>0.78</v>
+        <v>40000000</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="8">
-        <v>40000000</v>
-      </c>
+      <c r="A15" s="7"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="7"/>
@@ -2899,9 +2855,6 @@
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A70" s="7"/>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A71" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2935,41 +2888,41 @@
     </row>
     <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>36</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B3">
         <v>0</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B4" s="11" t="s">
         <v>51</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>23</v>
@@ -2977,27 +2930,27 @@
     </row>
     <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>34</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>22</v>
@@ -3005,7 +2958,7 @@
     </row>
     <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B7" s="11">
         <v>1</v>
@@ -3014,12 +2967,12 @@
         <v>48</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B8" s="11">
         <v>0</v>
@@ -3028,15 +2981,15 @@
         <v>47</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>51</v>
@@ -3047,13 +3000,13 @@
     </row>
     <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>22</v>
@@ -3064,10 +3017,10 @@
         <v>25</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>22</v>
@@ -3075,13 +3028,13 @@
     </row>
     <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>52</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>23</v>
@@ -3089,49 +3042,49 @@
     </row>
     <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>37</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B16" s="11" t="s">
         <v>44</v>
@@ -3140,18 +3093,18 @@
         <v>43</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>22</v>
@@ -3159,55 +3112,55 @@
     </row>
     <row r="18" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>22</v>
@@ -3215,13 +3168,13 @@
     </row>
     <row r="22" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D22" s="11" t="s">
         <v>22</v>
@@ -3229,27 +3182,27 @@
     </row>
     <row r="23" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>37</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>22</v>
@@ -3257,10 +3210,10 @@
     </row>
     <row r="25" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>37</v>
@@ -3271,41 +3224,41 @@
     </row>
     <row r="26" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B26">
         <v>0</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>35</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>22</v>
@@ -3313,10 +3266,10 @@
     </row>
     <row r="29" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>35</v>
@@ -3327,80 +3280,80 @@
     </row>
     <row r="30" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B30">
         <v>0</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B33">
         <v>0</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>46</v>
@@ -3411,10 +3364,10 @@
     </row>
     <row r="36" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>46</v>
@@ -3425,10 +3378,10 @@
     </row>
     <row r="37" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>44</v>
@@ -3439,10 +3392,10 @@
     </row>
     <row r="38" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>45</v>
@@ -3453,10 +3406,10 @@
     </row>
     <row r="39" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>45</v>
@@ -3467,10 +3420,10 @@
     </row>
     <row r="40" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>43</v>
@@ -3481,10 +3434,10 @@
     </row>
     <row r="41" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C41" s="11" t="s">
         <v>42</v>
@@ -3495,38 +3448,38 @@
     </row>
     <row r="42" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B43">
         <v>0</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C44" s="11" t="s">
         <v>54</v>
@@ -3540,7 +3493,7 @@
         <v>29</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C45" s="11" t="s">
         <v>54</v>
@@ -3551,13 +3504,13 @@
     </row>
     <row r="46" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C46" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D46" s="11" t="s">
         <v>22</v>
@@ -3568,13 +3521,13 @@
         <v>26</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -3582,13 +3535,13 @@
         <v>26</v>
       </c>
       <c r="B48" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C48" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="C48" s="11" t="s">
-        <v>99</v>
-      </c>
       <c r="D48" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -3596,13 +3549,13 @@
         <v>26</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -3610,13 +3563,13 @@
         <v>27</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -3627,15 +3580,15 @@
         <v>0</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B52" s="11">
         <v>1</v>
@@ -3644,7 +3597,7 @@
         <v>27</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -3652,7 +3605,7 @@
         <v>28</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C53" s="11" t="s">
         <v>54</v>
@@ -3669,10 +3622,10 @@
         <v>0</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -3683,7 +3636,7 @@
         <v>28</v>
       </c>
       <c r="C55" s="15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D55" s="15" t="s">
         <v>22</v>
@@ -3691,7 +3644,7 @@
     </row>
     <row r="56" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>27</v>
@@ -3700,7 +3653,7 @@
         <v>53</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -3708,10 +3661,10 @@
         <v>30</v>
       </c>
       <c r="B57" s="15" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C57" s="15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D57" s="15" t="s">
         <v>22</v>
@@ -3719,7 +3672,7 @@
     </row>
     <row r="58" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A58" s="15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B58" s="15" t="s">
         <v>55</v>
@@ -3728,12 +3681,12 @@
         <v>30</v>
       </c>
       <c r="D58" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B59" s="15">
         <v>1</v>
@@ -3742,32 +3695,32 @@
         <v>55</v>
       </c>
       <c r="D59" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A60" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B60" s="15">
         <v>1</v>
       </c>
       <c r="C60" s="15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D60" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B61" s="15" t="s">
         <v>55</v>
       </c>
       <c r="C61" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D61" s="15" t="s">
         <v>22</v>
@@ -3775,13 +3728,13 @@
     </row>
     <row r="62" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B62" s="15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C62" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D62" s="15" t="s">
         <v>22</v>
@@ -3789,13 +3742,13 @@
     </row>
     <row r="63" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A63" s="15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B63" s="15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C63" s="15" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D63" s="15" t="s">
         <v>22</v>
@@ -3803,13 +3756,13 @@
     </row>
     <row r="64" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A64" s="15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B64" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C64" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D64" s="15" t="s">
         <v>22</v>
@@ -3820,27 +3773,27 @@
         <v>31</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C65" s="15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D65" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C66" s="11">
         <v>0</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -3848,10 +3801,10 @@
         <v>32</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D67" s="11" t="s">
         <v>22</v>
@@ -3865,7 +3818,7 @@
         <v>0</v>
       </c>
       <c r="C68" s="15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D68" s="15" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
fix in DSM case
Changed ivi % RECs from 0 to 50 in dmo Partner RE, according to the book

Co-authored-by: Thom-Ivar <138502953+thomivarvandijk@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/src/vlinder/data/DSM/xlsx/DSM.xlsx
+++ b/src/vlinder/data/DSM/xlsx/DSM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tdijk004/Documents/Tooling/vlinder/trbs/src/vlinder/data/DSM/xlsx/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lheringa001/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{114CF110-45FB-9346-9CA8-CB0A11CEA40D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60416EDF-AEBC-404A-9C05-6A69215E5B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19800" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19800" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="configurations" sheetId="1" r:id="rId1"/>
@@ -584,8 +584,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
@@ -745,7 +745,7 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="23">
@@ -782,7 +782,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -808,9 +808,9 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Komma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{AE53C5E1-75E6-4245-B0B1-466E5639B5C7}"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -2194,7 +2194,7 @@
         <v>41</v>
       </c>
       <c r="C34" s="5">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>